<commit_message>
fix: Correct additional caratteristica values with fixed page matching
Fixed page format matching (112-113 vs 112 - 113) to catch 9 more corrections:

- C721: Peso max anta / 800 Kg / Velocità max / 18 m/min.
- 884 MC 3PH: Peso max anta / 3.500 Kg / Velocità max / 10 m/min
- D600: Forza max tiro/spinta
</commit_message>
<xml_diff>
--- a/output/v2/Data_Elena_P_KIT_v5_spaces_caratteristiche.xlsx
+++ b/output/v2/Data_Elena_P_KIT_v5_spaces_caratteristiche.xlsx
@@ -6342,22 +6342,22 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Larghezza max anta</t>
+          <t>Peso max anta</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>15 m</t>
+          <t>800 Kg</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>Velocità dell'anta</t>
+          <t>Velocità max</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>18 m/min (regolabile)</t>
+          <t>18 m/min.</t>
         </is>
       </c>
       <c r="O53" t="inlineStr"/>
@@ -7534,22 +7534,22 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>Larghezza max anta</t>
+          <t>Peso max anta</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>42 m</t>
+          <t>3.500 Kg</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>Peso max anta</t>
+          <t>Velocità max</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>3.500 Kg</t>
+          <t>10 m/min</t>
         </is>
       </c>
       <c r="O63" t="inlineStr"/>
@@ -7746,7 +7746,7 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>Forza max di spinta</t>
+          <t>Forza max tiro/spinta</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">

</xml_diff>

<commit_message>
fix: Correct badge_sistemi format with complete component descriptions
Updated S418, 412, 413 230V, 415 230V with correct format:
- Safe|<b>Sistema XXV SAFEzone:</b><br>PRODUCT + COMPONENTS
- Green|<b>Sistema XXV GREENtech:</b></br>PRODUCT + COMPONENTS

Previously missing <br> line breaks and component descriptions.
</commit_message>
<xml_diff>
--- a/output/v2/Data_Elena_P_KIT_v5_spaces_caratteristiche.xlsx
+++ b/output/v2/Data_Elena_P_KIT_v5_spaces_caratteristiche.xlsx
@@ -4188,7 +4188,7 @@
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;Sistema 24V SAFEzone:&lt;/b&gt;;Green</t>
+          <t>Safe|&lt;b&gt;Sistema 24V SAFEzone:&lt;/b&gt;&lt;br&gt;S418 + E024S o E124S;Green|&lt;b&gt;Sistema 24V GREENtech:&lt;/b&gt;&lt;/br&gt;S418 + E124S</t>
         </is>
       </c>
       <c r="T35" t="inlineStr"/>
@@ -4305,8 +4305,7 @@
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt; Sistema 230V SAFEzone:&lt;/b&gt;&lt;br&gt; 412 + E045S o E145S
-+ SAFEcoder;Green|&lt;b&gt;Sistema 230V GREENtech:&lt;/b&gt;</t>
+          <t>Safe|&lt;b&gt;Sistema 230V SAFEzone:&lt;/b&gt;&lt;br&gt;412 + E045S o E145S + SAFEcoder;Green|&lt;b&gt;Sistema 230V GREENtech:&lt;/b&gt;&lt;/br&gt;412 + E045S o E145S</t>
         </is>
       </c>
       <c r="T36" t="inlineStr"/>
@@ -4425,7 +4424,7 @@
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;Sistema 230V SAFEzone:&lt;/b&gt;;Green</t>
+          <t>Safe|&lt;b&gt;Sistema 230V SAFEzone:&lt;/b&gt;&lt;br&gt;413 230V + E045S o E145S + SAFEcoder</t>
         </is>
       </c>
       <c r="T37" t="inlineStr"/>
@@ -4543,7 +4542,7 @@
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;SAFEcoder encoder assoluto magnetico BUS&lt;/b&gt;;Green</t>
+          <t>Safe|&lt;b&gt;Sistema 230V SAFEzone:&lt;/b&gt;&lt;br&gt;415 230V + E045S o E145S + SAFEcoder</t>
         </is>
       </c>
       <c r="T38" t="inlineStr"/>

</xml_diff>

<commit_message>
fix: Complete badge_sistemi phrases with GREENtech components
Added missing GREENtech component descriptions for:
- 413 230V: +Green|<b>Sistema 230V GREENtech:</b></br>413 230V + E045S o E145S
- 415 230V: +Green|<b>Sistema 230V GREENtech:</b></br>415 230V + E045S o E145S
- 415 24V: Complete SAFEzone + GREENtech phrases
</commit_message>
<xml_diff>
--- a/output/v2/Data_Elena_P_KIT_v5_spaces_caratteristiche.xlsx
+++ b/output/v2/Data_Elena_P_KIT_v5_spaces_caratteristiche.xlsx
@@ -4424,7 +4424,7 @@
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;Sistema 230V SAFEzone:&lt;/b&gt;&lt;br&gt;413 230V + E045S o E145S + SAFEcoder</t>
+          <t>Safe|&lt;b&gt;Sistema 230V SAFEzone:&lt;/b&gt;&lt;br&gt;413 230V + E045S o E145S + SAFEcoder;Green|&lt;b&gt;Sistema 230V GREENtech:&lt;/b&gt;&lt;/br&gt;413 230V + E045S o E145S</t>
         </is>
       </c>
       <c r="T37" t="inlineStr"/>
@@ -4542,7 +4542,7 @@
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;Sistema 230V SAFEzone:&lt;/b&gt;&lt;br&gt;415 230V + E045S o E145S + SAFEcoder</t>
+          <t>Safe|&lt;b&gt;Sistema 230V SAFEzone:&lt;/b&gt;&lt;br&gt;415 230V + E045S o E145S + SAFEcoder;Green|&lt;b&gt;Sistema 230V GREENtech:&lt;/b&gt;&lt;/br&gt;415 230V + E045S o E145S</t>
         </is>
       </c>
       <c r="T38" t="inlineStr"/>
@@ -4663,7 +4663,7 @@
       <c r="R39" t="inlineStr"/>
       <c r="S39" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;Sistema 24V SAFEzone:&lt;/b&gt;;Green</t>
+          <t>Safe|&lt;b&gt;Sistema 24V SAFEzone:&lt;/b&gt;&lt;br&gt;415 24V + E024S o E124S;Green|&lt;b&gt;Sistema 24V GREENtech:&lt;/b&gt;&lt;/br&gt;415 24V + E124S</t>
         </is>
       </c>
       <c r="T39" t="inlineStr"/>

</xml_diff>

<commit_message>
fix: Complete badge_sistemi extraction from IDML
- Fixed LEADER kit (page 28): proper </b> placement after title
- Fixed LEADER kit (page 44): added component description
- Fixed 390 230V (page 82-83): added component description
- Fixed 770N 24V, S800H ENC, 560: complete phrases from IDML

Format: Safe|<b>Title:</b><br>Components;Green|<b>Title:</b></br>Components
</commit_message>
<xml_diff>
--- a/output/v2/Data_Elena_P_KIT_v5_spaces_caratteristiche.xlsx
+++ b/output/v2/Data_Elena_P_KIT_v5_spaces_caratteristiche.xlsx
@@ -872,8 +872,7 @@
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;SAFEzone composto da:  -LEADER kit230V + 2SAFEcoder (da acquistare separatamente)&lt;/b&gt;</t>
+          <t>Safe|&lt;b&gt;SAFEzone composto da:&lt;/b&gt;&lt;br&gt;LEADER kit230V + 2SAFEcoder (da acquistare separatamente)</t>
         </is>
       </c>
       <c r="T3" t="inlineStr"/>
@@ -2306,7 +2305,7 @@
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;SAFEzone composto da:&lt;/b&gt;</t>
+          <t>Safe|&lt;b&gt;SAFEzone composto da:&lt;/b&gt;&lt;br&gt;Leader kit 230V</t>
         </is>
       </c>
       <c r="T17" t="inlineStr"/>
@@ -4773,7 +4772,7 @@
       <c r="R40" t="inlineStr"/>
       <c r="S40" t="inlineStr">
         <is>
-          <t>Green|&lt;b&gt;Sistema 230V GREENtech:&lt;/b&gt;</t>
+          <t>Green|&lt;b&gt;Sistema 230V GREENtech:&lt;/b&gt;&lt;/br&gt;390 230V + E045S o E145S</t>
         </is>
       </c>
       <c r="T40" t="inlineStr"/>
@@ -5754,7 +5753,7 @@
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;Sistema 24V SAFEzone:&lt;/b&gt;;Green</t>
+          <t>Safe|&lt;b&gt;Sistema 24V SAFEzone:&lt;/b&gt;&lt;br&gt;770N 24V + E024S o E124S;Green|&lt;b&gt;Sistema 24V GREENtech:&lt;/b&gt;&lt;/br&gt;770N 24V + E124S</t>
         </is>
       </c>
       <c r="T48" t="inlineStr"/>
@@ -5879,7 +5878,7 @@
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;Sistema 24V SAFEzone:&lt;/b&gt;;Green</t>
+          <t>Safe|&lt;b&gt;Sistema 24V SAFEzone:&lt;/b&gt;&lt;br&gt;S800H ENC + E024S o E124S;Green|&lt;b&gt;Sistema 24V GREENtech:&lt;/b&gt;&lt;/br&gt;S800H ENC + E124S</t>
         </is>
       </c>
       <c r="T49" t="inlineStr"/>
@@ -8353,7 +8352,7 @@
       <c r="R70" t="inlineStr"/>
       <c r="S70" t="inlineStr">
         <is>
-          <t>Green|&lt;b&gt;Sistema 230V GREENtech:&lt;/b&gt;</t>
+          <t>Green|&lt;b&gt;Sistema 230V GREENtech:&lt;/b&gt;&lt;/br&gt;390 230V + E045S o E145S</t>
         </is>
       </c>
       <c r="T70" t="inlineStr"/>
@@ -8466,7 +8465,7 @@
       <c r="R71" t="inlineStr"/>
       <c r="S71" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>Green|&lt;b&gt;Sistema GREENtech:&lt;/b&gt;&lt;/br&gt;560 + E045S o E145S</t>
         </is>
       </c>
       <c r="T71" t="inlineStr"/>

</xml_diff>

<commit_message>
fix: Complete all badge_sistemi with full IDML data
Updated 16 products with complete badge phrases from IDML:
- 392 C: Green|<b>Sistema GREENtech:</b></br>392 24V + E034
- 402, 422, 400: Complete Safe + Green with components
- S2500I, 770N 230V: Added missing component descriptions
- Kit products: Fixed format and descriptions

Format: Type|<b>Title:</b><br>Components
</commit_message>
<xml_diff>
--- a/output/v2/Data_Elena_P_KIT_v5_spaces_caratteristiche.xlsx
+++ b/output/v2/Data_Elena_P_KIT_v5_spaces_caratteristiche.xlsx
@@ -971,8 +971,7 @@
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;SAFEzone composto da:  -LEADER kit230V + 2SAFEcoder (da acquistare separatamente)&lt;/b&gt;</t>
+          <t>Safe|&lt;b&gt;SAFEzone composto da:&lt;/b&gt;&lt;br&gt;MASTER kit230V + 2SAFEcoder (da acquistare separatamente)</t>
         </is>
       </c>
       <c r="T4" t="inlineStr"/>
@@ -1481,7 +1480,7 @@
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;SAFEzone composto da: POWER kit230V + 2SAFEcoder (da acquistare separatamente)&lt;/b&gt;</t>
+          <t>Safe|&lt;b&gt;SAFEzone composto da:&lt;/b&gt;&lt;br&gt;POWER kit230V + 2SAFEcoder (da acquistare separatamente)</t>
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
@@ -1588,7 +1587,7 @@
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;SAFEzone composto da: POWER kit230V + 2SAFEcoder (da acquistare separatamente)&lt;/b&gt;</t>
+          <t>Safe|&lt;b&gt;SAFEzone composto da:&lt;/b&gt;&lt;br&gt;POWER kit230V + 2SAFEcoder (da acquistare separatamente)</t>
         </is>
       </c>
       <c r="T10" t="inlineStr"/>
@@ -2404,7 +2403,7 @@
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;SAFEzone composto da:&lt;/b&gt;</t>
+          <t>Safe|&lt;b&gt;SAFEzone composto da:&lt;/b&gt;&lt;br&gt;Trendy kit 230V</t>
         </is>
       </c>
       <c r="T18" t="inlineStr"/>
@@ -2503,7 +2502,7 @@
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;SAFEzone composto da:&lt;/b&gt;</t>
+          <t>Safe|&lt;b&gt;SAFEzone composto da:&lt;/b&gt;&lt;br&gt;MASTER kit 230V</t>
         </is>
       </c>
       <c r="T19" t="inlineStr"/>
@@ -2602,7 +2601,7 @@
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;La confezione MASTER kit 24V SAFE comprende:&lt;/b&gt;</t>
+          <t>Safe|&lt;b&gt;SAFEzone composto da:&lt;/b&gt;&lt;br&gt;MASTER kit 230V</t>
         </is>
       </c>
       <c r="T20" t="inlineStr"/>
@@ -2701,7 +2700,7 @@
       <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;SAFEcoder per attuatore 412 (&lt;/b&gt;</t>
+          <t>Safe|&lt;b&gt;SAFEzone composto da:&lt;/b&gt;&lt;br&gt;ECO kit 230V</t>
         </is>
       </c>
       <c r="T21" t="inlineStr"/>
@@ -2800,7 +2799,7 @@
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;SAFEcoder per attuatore 412 (&lt;/b&gt;</t>
+          <t>Safe|&lt;b&gt;SAFEzone composto da:&lt;/b&gt;&lt;br&gt;ECO kit 230V</t>
         </is>
       </c>
       <c r="T22" t="inlineStr"/>
@@ -3107,7 +3106,7 @@
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;POWER kit 24V SAFE&lt;/b&gt;</t>
+          <t>Safe|&lt;b&gt;SAFEzone composto da:&lt;/b&gt;&lt;br&gt;POWER kit 230V</t>
         </is>
       </c>
       <c r="T25" t="inlineStr"/>
@@ -3214,7 +3213,7 @@
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;POWER kit 24V SAFE&lt;/b&gt;</t>
+          <t>Safe|&lt;b&gt;SAFEzone composto da:&lt;/b&gt;&lt;br&gt;POWER kit 230V</t>
         </is>
       </c>
       <c r="T26" t="inlineStr"/>
@@ -4891,7 +4890,7 @@
       <c r="R41" t="inlineStr"/>
       <c r="S41" t="inlineStr">
         <is>
-          <t>Safe;Green|&lt;b&gt;Sistema GREENtech:&lt;/b&gt;</t>
+          <t>Green|&lt;b&gt;Sistema GREENtech:&lt;/b&gt;&lt;/br&gt;392 24V + E034</t>
         </is>
       </c>
       <c r="T41" t="inlineStr"/>
@@ -5027,7 +5026,7 @@
       <c r="R42" t="inlineStr"/>
       <c r="S42" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;Sistema SAFEzone:&lt;/b&gt;&lt;br&gt;402 + E045S o E145S + SAFEcoder green|&lt;b&gt;Sistema GREENtech:&lt;/b&gt;&lt;/br&gt; 402 + E045S o E145S;Green|&lt;b&gt;Sistema GREENtech:&lt;/b&gt;</t>
+          <t>Safe|&lt;b&gt;Sistema SAFEzone:&lt;/b&gt;&lt;br&gt;402 + E045S o E145S + SAFEcoder;Green|&lt;b&gt;Sistema GREENtech:&lt;/b&gt;&lt;/br&gt;402 + E045S o E145S</t>
         </is>
       </c>
       <c r="T42" t="inlineStr"/>
@@ -5149,8 +5148,7 @@
       <c r="R43" t="inlineStr"/>
       <c r="S43" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt; Sistema 230V SAFEzone: &lt;/b&gt;&lt;br&gt; 422 + E045S o E145S
-+ SAFEcoder;Green|&lt;b&gt;Sistema 230V GREENtech:&lt;/b&gt;</t>
+          <t>Safe|&lt;b&gt;Sistema 230V SAFEzone:&lt;/b&gt;&lt;br&gt;422 + E045S o E145S + SAFEcoder;Green|&lt;b&gt;Sistema 230V GREENtech:&lt;/b&gt;&lt;/br&gt;422 + E045S o E145S</t>
         </is>
       </c>
       <c r="T43" t="inlineStr"/>
@@ -5257,7 +5255,7 @@
       <c r="R44" t="inlineStr"/>
       <c r="S44" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;Sistema 230V SAFEzone:&lt;/b&gt;&lt;/br&gt; 400 + E045S o E145S + SAFEcoder;Green|&lt;b&gt;Sistema 230V GREENtech:&lt;/b&gt;</t>
+          <t>Safe|&lt;b&gt;Sistema 230V SAFEzone:&lt;/b&gt;&lt;br&gt;400 + E045S o E145S + SAFEcoder;Green|&lt;b&gt;Sistema 230V GREENtech:&lt;/b&gt;&lt;/br&gt;400 + E045S o E145S</t>
         </is>
       </c>
       <c r="T44" t="inlineStr"/>
@@ -5504,7 +5502,7 @@
       <c r="R46" t="inlineStr"/>
       <c r="S46" t="inlineStr">
         <is>
-          <t>Safe|&lt;b&gt;Sistema 24V SAFEzone:&lt;/b&gt;;Green|&lt;b&gt;Sistema 24V GREENtech:&lt;/b&gt;</t>
+          <t>Safe|&lt;b&gt;Sistema 24V SAFEzone:&lt;/b&gt;&lt;br&gt;S2500I + E124S;Green|&lt;b&gt;Sistema 24V GREENtech:&lt;/b&gt;&lt;/br&gt;S2500I + E124S</t>
         </is>
       </c>
       <c r="T46" t="inlineStr">
@@ -5627,7 +5625,7 @@
       <c r="R47" t="inlineStr"/>
       <c r="S47" t="inlineStr">
         <is>
-          <t>Safe;Green</t>
+          <t>Safe|&lt;b&gt;Sistema 230V SAFEzone:&lt;/b&gt;&lt;br&gt;770N 230V + E045S o E145S + SAFEcoder;Green|&lt;b&gt;Sistema 230V GREENtech:&lt;/b&gt;&lt;/br&gt;770N 230V + E045S o E145S</t>
         </is>
       </c>
       <c r="T47" t="inlineStr"/>

</xml_diff>